<commit_message>
Changes on code to generate and run the DDD api test cases yaml file
</commit_message>
<xml_diff>
--- a/input/api/DEP_App_Dashboard_DDD_API_Design_v1.3.xlsx
+++ b/input/api/DEP_App_Dashboard_DDD_API_Design_v1.3.xlsx
@@ -16517,10 +16517,10 @@
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="88ca0028-d944-4b54-a24a-33c956642033">
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb43bdf0-3619-4b54-b31e-a8a72f171391">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aef3f498-749b-43cd-ac3b-f8654dcba8c2" xsi:nil="true"/>
+    <TaxCatchAll xmlns="2dadf7ee-14cc-45f3-948a-a38a0e838d24" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
@@ -16535,10 +16535,10 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005A3C49B5B8A2D749BAFDCDB853B21597" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0f0958eff6a3a4a206dce48da463fc29">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="88ca0028-d944-4b54-a24a-33c956642033" xmlns:ns3="aef3f498-749b-43cd-ac3b-f8654dcba8c2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d362f1f0b652b2f2d438f5707b209cbb" ns2:_="" ns3:_="">
-    <xsd:import namespace="88ca0028-d944-4b54-a24a-33c956642033"/>
-    <xsd:import namespace="aef3f498-749b-43cd-ac3b-f8654dcba8c2"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A9B4981540F375498654EAFF3F046281" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8a5ebea04648d29e8f47710243b77275">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eb43bdf0-3619-4b54-b31e-a8a72f171391" xmlns:ns3="2dadf7ee-14cc-45f3-948a-a38a0e838d24" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d8d4f3bc4cf75db31872049f5cbc23a" ns2:_="" ns3:_="">
+    <xsd:import namespace="eb43bdf0-3619-4b54-b31e-a8a72f171391"/>
+    <xsd:import namespace="2dadf7ee-14cc-45f3-948a-a38a0e838d24"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -16555,7 +16555,6 @@
                 <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
                 <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -16563,7 +16562,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="88ca0028-d944-4b54-a24a-33c956642033" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="eb43bdf0-3619-4b54-b31e-a8a72f171391" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -16615,16 +16614,11 @@
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="aef3f498-749b-43cd-ac3b-f8654dcba8c2" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2dadf7ee-14cc-45f3-948a-a38a0e838d24" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{cdc93b2a-8661-4444-939a-2cf5c9f51721}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="aef3f498-749b-43cd-ac3b-f8654dcba8c2">
+    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{bc5e150e-238a-448e-9cab-ff45677664b7}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2dadf7ee-14cc-45f3-948a-a38a0e838d24">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -16761,22 +16755,7 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1330EDBE-8A3A-40C3-BED1-F87695A5C4ED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="88ca0028-d944-4b54-a24a-33c956642033"/>
-    <ds:schemaRef ds:uri="aef3f498-749b-43cd-ac3b-f8654dcba8c2"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9519EAC8-3C7A-4580-82EF-1777877CBB4A}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>